<commit_message>
Personalize portfolio with Saw Oo Lin's real academic and work data
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -428,7 +428,7 @@
         <v>Projects</v>
       </c>
       <c r="B3" t="str">
-        <v>5+</v>
+        <v>3+</v>
       </c>
       <c r="C3" t="str">
         <v>Major Projects</v>
@@ -469,7 +469,7 @@
         <v>p1</v>
       </c>
       <c r="B2" t="str">
-        <v>I am a highly motivated scholarship student pursuing a degree in Computer Science. My goal is to leverage my academic background to drive positive impact in the tech industry.</v>
+        <v>I am a highly motivated student pursuing a Bachelor of Science in Software Development. My goal is to leverage my academic background to drive positive impact in the tech industry.</v>
       </c>
     </row>
     <row r="3">
@@ -477,7 +477,7 @@
         <v>p2</v>
       </c>
       <c r="B3" t="str">
-        <v>Through various leadership roles and academic excellence, I have proven my dedication to continuous learning and community engagement.</v>
+        <v>Through various leadership roles and academic excellence across multiple institutions, I have proven my dedication to continuous learning and community engagement.</v>
       </c>
     </row>
   </sheetData>
@@ -510,13 +510,13 @@
         <v>Academics</v>
       </c>
       <c r="B2" t="str">
-        <v>Dean's Excellence Scholarship</v>
+        <v>American University of Phnom Penh (AUPP)</v>
       </c>
       <c r="C2" t="str">
-        <v>2023 - Present</v>
+        <v>Aug 2024 - Present</v>
       </c>
       <c r="D2" t="str">
-        <v>Awarded for outstanding academic performance and leadership potential among incoming freshmen.</v>
+        <v>Bachelor of Science in Software Development</v>
       </c>
     </row>
     <row r="3">
@@ -524,27 +524,27 @@
         <v>Academics</v>
       </c>
       <c r="B3" t="str">
-        <v>National Science Fair - 1st Place</v>
+        <v>TOUNGE LA' YAT COMMUNITY COLLEGE</v>
       </c>
       <c r="C3" t="str">
-        <v>2022</v>
+        <v>Jan 2022 - Dec 2023</v>
       </c>
       <c r="D3" t="str">
-        <v>Developed an AI model predicting crop yields to assist local farmers, winning top honors nationally.</v>
+        <v>Diploma in Social and Development Studies</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Experience</v>
+        <v>Academics</v>
       </c>
       <c r="B4" t="str">
-        <v>Software Engineering Intern</v>
+        <v>University of Yangon</v>
       </c>
       <c r="C4" t="str">
-        <v>Summer 2023</v>
+        <v>Dec 2018 - Mar 2020</v>
       </c>
       <c r="D4" t="str">
-        <v>Assisted in the backend development of a scalable REST API using Node.js and improved database query performance by 20%.</v>
+        <v>Bachelor of Science in Mathematics (2nd yr, incomplete)</v>
       </c>
     </row>
     <row r="5">
@@ -552,13 +552,13 @@
         <v>Experience</v>
       </c>
       <c r="B5" t="str">
-        <v>Past Community Development Leader</v>
+        <v>Junior Associate, Operations</v>
       </c>
       <c r="C5" t="str">
-        <v>2020 - 2022</v>
+        <v>June 2025 - Present</v>
       </c>
       <c r="D5" t="str">
-        <v>Spearheaded local neighborhood revitalization projects, organizing over 200 volunteers for after-school mentorship programs and community gardening.</v>
+        <v>AUPP Technology Center (ATC)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>